<commit_message>
feat: SpaceX Valuation Analysis — Task 3 (initiating coverage)
繁體中文估值分析 (20KB)：DCF退出乘數法、可比公司分析（8家）、
分部加總法（SOTP），目標股價 $205，較假設 IPO 價格 $152 具 34.9%
上行空間；評級：買入（BUY/OUTPERFORM）。

Excel 財務模型新增 5 個估值標籤頁（共 11 頁）：
DCF Analysis | Sensitivity Analysis | Comparable Companies |
Valuation Summary | SOTP Analysis

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/spacex-initiation-coverage/SpaceX_Financial_Model_2026-05-24.xlsx
+++ b/spacex-initiation-coverage/SpaceX_Financial_Model_2026-05-24.xlsx
@@ -13,6 +13,11 @@
     <sheet name="Balance Sheet" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="Scenarios" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="DCF Inputs" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="DCF Analysis" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Sensitivity Analysis" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Comparable Companies" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Valuation Summary" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="SOTP Analysis" sheetId="11" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -21,12 +26,16 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="3">
+  <numFmts count="7">
     <numFmt numFmtId="164" formatCode="0.0%"/>
     <numFmt numFmtId="165" formatCode="$0.00"/>
     <numFmt numFmtId="166" formatCode="#,##0.0"/>
+    <numFmt numFmtId="167" formatCode="0.0000"/>
+    <numFmt numFmtId="168" formatCode="&quot;$&quot;#,##0"/>
+    <numFmt numFmtId="169" formatCode="0.0&quot;x&quot;"/>
+    <numFmt numFmtId="170" formatCode="&quot;$&quot;#,##0.0"/>
   </numFmts>
-  <fonts count="22">
+  <fonts count="25">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -152,8 +161,24 @@
       <name val="Calibri"/>
       <sz val="8"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <i val="1"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="000070C0"/>
+      <sz val="9"/>
+    </font>
   </fonts>
-  <fills count="11">
+  <fills count="14">
     <fill>
       <patternFill/>
     </fill>
@@ -205,6 +230,21 @@
         <fgColor rgb="00FCE4D6"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C6EFCE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FDDCBD"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F2F2F2"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="4">
     <border>
@@ -235,7 +275,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="63">
+  <cellXfs count="108">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -419,6 +459,135 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="164" fontId="4" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="3" fontId="5" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="7" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="168" fontId="5" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="5" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="5" fillId="11" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="5" fillId="12" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="7" fillId="12" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="7" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="7" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="7" fillId="11" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="5" fillId="10" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="169" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="7" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="169" fontId="7" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="13" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="169" fontId="5" fillId="13" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="13" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="169" fontId="7" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="170" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="7" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="7" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
   </cellXfs>
@@ -2961,6 +3130,821 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="00843C0C"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="B1:G28"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="2" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="26" customHeight="1">
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>SpaceX (SPCE)  —  估值摘要與建議</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="13" customHeight="1">
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>加權平均法；目標股價 = $205；假設 IPO 股價 = $152；金額：美元每股</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="5" customHeight="1"/>
+    <row r="5">
+      <c r="B5" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  估值方法匯總</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="B6" s="63" t="inlineStr">
+        <is>
+          <t>估值方法</t>
+        </is>
+      </c>
+      <c r="C6" s="63" t="inlineStr">
+        <is>
+          <t>每股估值（低）</t>
+        </is>
+      </c>
+      <c r="D6" s="63" t="inlineStr">
+        <is>
+          <t>每股估值（基準）</t>
+        </is>
+      </c>
+      <c r="E6" s="63" t="inlineStr">
+        <is>
+          <t>每股估值（高）</t>
+        </is>
+      </c>
+      <c r="F6" s="63" t="inlineStr">
+        <is>
+          <t>權重</t>
+        </is>
+      </c>
+      <c r="G6" s="63" t="inlineStr">
+        <is>
+          <t>加權貢獻</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="16" customHeight="1">
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  現金流折現法（DCF）</t>
+        </is>
+      </c>
+      <c r="C7" s="99" t="n">
+        <v>160</v>
+      </c>
+      <c r="D7" s="100" t="n">
+        <v>191.85</v>
+      </c>
+      <c r="E7" s="99" t="n">
+        <v>224</v>
+      </c>
+      <c r="F7" s="25" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="G7" s="101" t="n">
+        <v>76.73999999999999</v>
+      </c>
+    </row>
+    <row r="8" ht="16" customHeight="1">
+      <c r="B8" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  可比公司倍數法（Comps）</t>
+        </is>
+      </c>
+      <c r="C8" s="99" t="n">
+        <v>165</v>
+      </c>
+      <c r="D8" s="100" t="n">
+        <v>201.57</v>
+      </c>
+      <c r="E8" s="99" t="n">
+        <v>235</v>
+      </c>
+      <c r="F8" s="25" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="G8" s="101" t="n">
+        <v>70.55</v>
+      </c>
+    </row>
+    <row r="9" ht="16" customHeight="1">
+      <c r="B9" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  分部加總法（SOTP）</t>
+        </is>
+      </c>
+      <c r="C9" s="99" t="n">
+        <v>170</v>
+      </c>
+      <c r="D9" s="100" t="n">
+        <v>220.85</v>
+      </c>
+      <c r="E9" s="99" t="n">
+        <v>265</v>
+      </c>
+      <c r="F9" s="25" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="G9" s="101" t="n">
+        <v>55.21</v>
+      </c>
+    </row>
+    <row r="10" ht="18" customHeight="1">
+      <c r="B10" s="84" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  加權平均目標股價</t>
+        </is>
+      </c>
+      <c r="C10" s="76" t="n">
+        <v>160</v>
+      </c>
+      <c r="D10" s="76" t="n">
+        <v>202.5</v>
+      </c>
+      <c r="E10" s="76" t="n">
+        <v>265</v>
+      </c>
+      <c r="F10" s="89" t="n">
+        <v>1</v>
+      </c>
+      <c r="G10" s="102" t="n">
+        <v>202.5</v>
+      </c>
+    </row>
+    <row r="11" ht="8" customHeight="1"/>
+    <row r="12">
+      <c r="B12" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  最終投資建議</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="16" customHeight="1">
+      <c r="B13" s="24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  評級</t>
+        </is>
+      </c>
+      <c r="E13" s="103" t="inlineStr">
+        <is>
+          <t>買入（BUY / OUTPERFORM）</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="16" customHeight="1">
+      <c r="B14" s="24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  12個月目標股價</t>
+        </is>
+      </c>
+      <c r="E14" s="103" t="inlineStr">
+        <is>
+          <t>$205</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="16" customHeight="1">
+      <c r="B15" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  假設 IPO 股價</t>
+        </is>
+      </c>
+      <c r="E15" s="104" t="inlineStr">
+        <is>
+          <t>$152</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="16" customHeight="1">
+      <c r="B16" s="24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  潛在回報（資本增值）</t>
+        </is>
+      </c>
+      <c r="E16" s="103" t="inlineStr">
+        <is>
+          <t>34.9%</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="16" customHeight="1">
+      <c r="B17" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  企業價值（DCF 基準）</t>
+        </is>
+      </c>
+      <c r="E17" s="104" t="inlineStr">
+        <is>
+          <t>$321.4B</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="16" customHeight="1">
+      <c r="B18" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  市值（按 IPO 股價）</t>
+        </is>
+      </c>
+      <c r="E18" s="104" t="inlineStr">
+        <is>
+          <t>$322.2B</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="16" customHeight="1">
+      <c r="B19" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  攤薄股數</t>
+        </is>
+      </c>
+      <c r="E19" s="104" t="inlineStr">
+        <is>
+          <t>2,120M</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="16" customHeight="1">
+      <c r="B20" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  估值方法權重</t>
+        </is>
+      </c>
+      <c r="E20" s="104" t="inlineStr">
+        <is>
+          <t>DCF 40% | Comps 35% | SOTP 25%</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="8" customHeight="1"/>
+    <row r="22">
+      <c r="B22" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  分部加總細項</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="B23" s="63" t="inlineStr">
+        <is>
+          <t>業務部門</t>
+        </is>
+      </c>
+      <c r="C23" s="63" t="inlineStr">
+        <is>
+          <t>2027E收入($M)</t>
+        </is>
+      </c>
+      <c r="D23" s="63" t="inlineStr">
+        <is>
+          <t>收入佔比</t>
+        </is>
+      </c>
+      <c r="E23" s="63" t="inlineStr">
+        <is>
+          <t>應用倍數</t>
+        </is>
+      </c>
+      <c r="F23" s="63" t="inlineStr">
+        <is>
+          <t>隱含EV($B)</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="15" customHeight="1">
+      <c r="B24" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  太空發射服務</t>
+        </is>
+      </c>
+      <c r="C24" s="8" t="n">
+        <v>8208</v>
+      </c>
+      <c r="D24" s="25" t="n">
+        <v>0.216</v>
+      </c>
+      <c r="E24" s="81" t="n">
+        <v>3</v>
+      </c>
+      <c r="F24" s="80" t="n">
+        <v>24.62</v>
+      </c>
+    </row>
+    <row r="25" ht="15" customHeight="1">
+      <c r="B25" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Starlink 衛星連接</t>
+        </is>
+      </c>
+      <c r="C25" s="8" t="n">
+        <v>21812</v>
+      </c>
+      <c r="D25" s="25" t="n">
+        <v>0.574</v>
+      </c>
+      <c r="E25" s="81" t="n">
+        <v>8</v>
+      </c>
+      <c r="F25" s="80" t="n">
+        <v>174.5</v>
+      </c>
+    </row>
+    <row r="26" ht="15" customHeight="1">
+      <c r="B26" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  AI 與科技（xAI/Grok）</t>
+        </is>
+      </c>
+      <c r="C26" s="8" t="n">
+        <v>7296</v>
+      </c>
+      <c r="D26" s="25" t="n">
+        <v>0.192</v>
+      </c>
+      <c r="E26" s="81" t="n">
+        <v>25</v>
+      </c>
+      <c r="F26" s="80" t="n">
+        <v>182.4</v>
+      </c>
+    </row>
+    <row r="27" ht="15" customHeight="1">
+      <c r="B27" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  其他</t>
+        </is>
+      </c>
+      <c r="C27" s="8" t="n">
+        <v>684</v>
+      </c>
+      <c r="D27" s="25" t="n">
+        <v>0.018</v>
+      </c>
+      <c r="E27" s="81" t="n">
+        <v>2</v>
+      </c>
+      <c r="F27" s="80" t="n">
+        <v>1.37</v>
+      </c>
+    </row>
+    <row r="28" ht="16" customHeight="1">
+      <c r="B28" s="24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  合計 / 加回淨現金</t>
+        </is>
+      </c>
+      <c r="C28" s="28" t="n">
+        <v>38000</v>
+      </c>
+      <c r="D28" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="E28" s="105" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F28" s="106" t="n">
+        <v>382.89</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="5">
+    <mergeCell ref="B2:G2"/>
+    <mergeCell ref="B5:G5"/>
+    <mergeCell ref="B22:G22"/>
+    <mergeCell ref="B1:G1"/>
+    <mergeCell ref="B12:G12"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="00843C0C"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="B1:I22"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="2" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="26" customHeight="1">
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>SpaceX (SPCE)  —  分部加總估值（SOTP）</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="13" customHeight="1">
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>按三大業務部門分別應用可比倍數；NTM 基準年 = 2027E；金額：$M 除另有說明</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="B4" s="63" t="inlineStr">
+        <is>
+          <t>業務部門 / 指標</t>
+        </is>
+      </c>
+      <c r="C4" s="63" t="inlineStr">
+        <is>
+          <t>2026E 收入</t>
+        </is>
+      </c>
+      <c r="D4" s="63" t="inlineStr">
+        <is>
+          <t>2027E 收入</t>
+        </is>
+      </c>
+      <c r="E4" s="63" t="inlineStr">
+        <is>
+          <t>收入增長</t>
+        </is>
+      </c>
+      <c r="F4" s="63" t="inlineStr">
+        <is>
+          <t>EBITDA 利潤率</t>
+        </is>
+      </c>
+      <c r="G4" s="63" t="inlineStr">
+        <is>
+          <t>應用倍數</t>
+        </is>
+      </c>
+      <c r="H4" s="63" t="inlineStr">
+        <is>
+          <t>隱含 EV ($M)</t>
+        </is>
+      </c>
+      <c r="I4" s="63" t="inlineStr">
+        <is>
+          <t>應用倍數依據</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="15" customHeight="1">
+      <c r="B5" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  太空發射服務</t>
+        </is>
+      </c>
+      <c r="C5" s="27" t="n">
+        <v>6909.28</v>
+      </c>
+      <c r="D5" s="27" t="n">
+        <v>8208</v>
+      </c>
+      <c r="E5" s="17" t="n">
+        <v>-0.129</v>
+      </c>
+      <c r="F5" s="17" t="n">
+        <v>0.39</v>
+      </c>
+      <c r="G5" s="107" t="inlineStr">
+        <is>
+          <t>3.0x EV/Rev</t>
+        </is>
+      </c>
+      <c r="H5" s="27" t="n">
+        <v>24624</v>
+      </c>
+      <c r="I5" s="83" t="inlineStr">
+        <is>
+          <t>NOC/LMT 防禦航太中位數 1.8x，加 Starship 技術溢價</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="15" customHeight="1">
+      <c r="B6" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    政府發射</t>
+        </is>
+      </c>
+      <c r="C6" s="8" t="n">
+        <v>3420</v>
+      </c>
+      <c r="D6" s="8" t="n">
+        <v>3990</v>
+      </c>
+      <c r="E6" s="25" t="n">
+        <v>0.1667</v>
+      </c>
+    </row>
+    <row r="7" ht="15" customHeight="1">
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    商業發射</t>
+        </is>
+      </c>
+      <c r="C7" s="8" t="n">
+        <v>1860</v>
+      </c>
+      <c r="D7" s="8" t="n">
+        <v>2250</v>
+      </c>
+      <c r="E7" s="25" t="n">
+        <v>0.2097</v>
+      </c>
+    </row>
+    <row r="8" ht="15" customHeight="1">
+      <c r="B8" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    Starship商業任務</t>
+        </is>
+      </c>
+      <c r="C8" s="8" t="n">
+        <v>1620</v>
+      </c>
+      <c r="D8" s="8" t="n">
+        <v>1970</v>
+      </c>
+    </row>
+    <row r="9" ht="15" customHeight="1">
+      <c r="B9" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Starlink 衛星連接</t>
+        </is>
+      </c>
+      <c r="C9" s="27" t="n">
+        <v>16632.42</v>
+      </c>
+      <c r="D9" s="27" t="n">
+        <v>21812</v>
+      </c>
+      <c r="E9" s="17" t="n">
+        <v>-0.0385</v>
+      </c>
+      <c r="F9" s="17" t="n">
+        <v>0.52</v>
+      </c>
+      <c r="G9" s="107" t="inlineStr">
+        <is>
+          <t>8.0x EV/Rev</t>
+        </is>
+      </c>
+      <c r="H9" s="27" t="n">
+        <v>174496</v>
+      </c>
+      <c r="I9" s="83" t="inlineStr">
+        <is>
+          <t>Iridium 6.5x，加用戶增長及直連手機溢價</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="15" customHeight="1">
+      <c r="B10" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    消費者寬頻</t>
+        </is>
+      </c>
+      <c r="C10" s="8" t="n">
+        <v>11200</v>
+      </c>
+      <c r="D10" s="8" t="n">
+        <v>14600</v>
+      </c>
+      <c r="E10" s="25" t="n">
+        <v>0.3036</v>
+      </c>
+    </row>
+    <row r="11" ht="15" customHeight="1">
+      <c r="B11" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    海事+航空</t>
+        </is>
+      </c>
+      <c r="C11" s="8" t="n">
+        <v>2380</v>
+      </c>
+      <c r="D11" s="8" t="n">
+        <v>3030</v>
+      </c>
+    </row>
+    <row r="12" ht="15" customHeight="1">
+      <c r="B12" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    政府+直連手機</t>
+        </is>
+      </c>
+      <c r="C12" s="8" t="n">
+        <v>3060</v>
+      </c>
+      <c r="D12" s="8" t="n">
+        <v>4180</v>
+      </c>
+    </row>
+    <row r="13" ht="15" customHeight="1">
+      <c r="B13" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  AI 與科技（xAI / Grok）</t>
+        </is>
+      </c>
+      <c r="C13" s="27" t="n">
+        <v>3788.96</v>
+      </c>
+      <c r="D13" s="27" t="n">
+        <v>7296</v>
+      </c>
+      <c r="E13" s="17" t="n">
+        <v>0.4118</v>
+      </c>
+      <c r="F13" s="17" t="n">
+        <v>0.62</v>
+      </c>
+      <c r="G13" s="107" t="inlineStr">
+        <is>
+          <t>25.0x EV/Rev</t>
+        </is>
+      </c>
+      <c r="H13" s="27" t="n">
+        <v>182400</v>
+      </c>
+      <c r="I13" s="83" t="inlineStr">
+        <is>
+          <t>Palantir 28.6x 折讓，反映業務仍在整合初期</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="15" customHeight="1">
+      <c r="B14" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    Grok 訂閱+API</t>
+        </is>
+      </c>
+      <c r="C14" s="8" t="n">
+        <v>2100</v>
+      </c>
+      <c r="D14" s="8" t="n">
+        <v>3850</v>
+      </c>
+      <c r="E14" s="25" t="n">
+        <v>0.8333</v>
+      </c>
+    </row>
+    <row r="15" ht="15" customHeight="1">
+      <c r="B15" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    AI 算力服務</t>
+        </is>
+      </c>
+      <c r="C15" s="8" t="n">
+        <v>1050</v>
+      </c>
+      <c r="D15" s="8" t="n">
+        <v>2100</v>
+      </c>
+      <c r="E15" s="25" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16" ht="15" customHeight="1">
+      <c r="B16" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    AI 企業授權</t>
+        </is>
+      </c>
+      <c r="C16" s="8" t="n">
+        <v>650</v>
+      </c>
+      <c r="D16" s="8" t="n">
+        <v>1350</v>
+      </c>
+      <c r="E16" s="25" t="n">
+        <v>2.0769</v>
+      </c>
+    </row>
+    <row r="17" ht="15" customHeight="1">
+      <c r="B17" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  其他（維修/技術許可）</t>
+        </is>
+      </c>
+      <c r="C17" s="27" t="n">
+        <v>520</v>
+      </c>
+      <c r="D17" s="27" t="n">
+        <v>680</v>
+      </c>
+      <c r="E17" s="17" t="n">
+        <v>0.3077</v>
+      </c>
+      <c r="F17" s="17" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="G17" s="107" t="inlineStr">
+        <is>
+          <t>2.0x EV/Rev</t>
+        </is>
+      </c>
+      <c r="H17" s="27" t="n">
+        <v>1368</v>
+      </c>
+      <c r="I17" s="83" t="inlineStr">
+        <is>
+          <t>低增長、非核心業務</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="18" customHeight="1">
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  業務合計 EV（SOTP）</t>
+        </is>
+      </c>
+      <c r="C18" s="28" t="n">
+        <v>27850.66</v>
+      </c>
+      <c r="D18" s="28" t="n">
+        <v>38000</v>
+      </c>
+      <c r="H18" s="22" t="n">
+        <v>382888</v>
+      </c>
+    </row>
+    <row r="19" ht="15" customHeight="1">
+      <c r="B19" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  + 淨現金（2026E 末，含 IPO 募資）</t>
+        </is>
+      </c>
+      <c r="H19" s="8" t="n">
+        <v>85322.48</v>
+      </c>
+    </row>
+    <row r="20" ht="15" customHeight="1">
+      <c r="B20" s="24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  股票總值</t>
+        </is>
+      </c>
+      <c r="H20" s="27" t="n">
+        <v>468210.48</v>
+      </c>
+    </row>
+    <row r="21" ht="15" customHeight="1">
+      <c r="B21" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ÷ 攤薄股數（M）</t>
+        </is>
+      </c>
+      <c r="H21" s="8" t="n">
+        <v>2120</v>
+      </c>
+    </row>
+    <row r="22" ht="15" customHeight="1">
+      <c r="B22" s="24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  每股股價（SOTP）</t>
+        </is>
+      </c>
+      <c r="H22" s="100" t="n">
+        <v>220.85</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="B1:I1"/>
+    <mergeCell ref="B2:I2"/>
+    <mergeCell ref="B18"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
@@ -4837,13 +5821,13 @@
         </is>
       </c>
       <c r="C70" s="30" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="D70" s="30" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="E70" s="30" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="F70" s="30" t="n">
         <v>0</v>
@@ -4871,13 +5855,13 @@
         </is>
       </c>
       <c r="C71" s="30" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="D71" s="30" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="E71" s="30" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="F71" s="30" t="n">
         <v>0</v>
@@ -8583,4 +9567,1422 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="002F5496"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="B1:I40"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="2" customWidth="1" min="1" max="1"/>
+    <col width="32" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
+    <col width="13" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="26" customHeight="1">
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>SpaceX (SPCE)  —  現金流折現估值 (DCF)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="13" customHeight="1">
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>退出乘數法；WACC = 13.5%；退出倍數 = 18x 2030E EBITDA；金額單位：百萬美元（$M）</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="B4" s="63" t="inlineStr">
+        <is>
+          <t>項目</t>
+        </is>
+      </c>
+      <c r="C4" s="63" t="inlineStr">
+        <is>
+          <t>2026E</t>
+        </is>
+      </c>
+      <c r="D4" s="63" t="inlineStr">
+        <is>
+          <t>2027E</t>
+        </is>
+      </c>
+      <c r="E4" s="63" t="inlineStr">
+        <is>
+          <t>2028E</t>
+        </is>
+      </c>
+      <c r="F4" s="63" t="inlineStr">
+        <is>
+          <t>2029E</t>
+        </is>
+      </c>
+      <c r="G4" s="63" t="inlineStr">
+        <is>
+          <t>2030E</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="5" customHeight="1"/>
+    <row r="6">
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  WACC 計算</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="15" customHeight="1">
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  無風險利率（10年期美國國債）</t>
+        </is>
+      </c>
+      <c r="F7" s="58" t="n">
+        <v>0.043</v>
+      </c>
+    </row>
+    <row r="8" ht="15" customHeight="1">
+      <c r="B8" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  股票風險溢價（ERP）</t>
+        </is>
+      </c>
+      <c r="F8" s="58" t="n">
+        <v>0.055</v>
+      </c>
+    </row>
+    <row r="9" ht="15" customHeight="1">
+      <c r="B9" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  調整後Beta</t>
+        </is>
+      </c>
+      <c r="F9" s="64" t="n">
+        <v>1.65</v>
+      </c>
+    </row>
+    <row r="10" ht="15" customHeight="1">
+      <c r="B10" s="24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  股本成本</t>
+        </is>
+      </c>
+      <c r="F10" s="65" t="n">
+        <v>0.134</v>
+      </c>
+    </row>
+    <row r="11" ht="15" customHeight="1">
+      <c r="B11" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  稅前債務成本</t>
+        </is>
+      </c>
+      <c r="F11" s="58" t="n">
+        <v>0.058</v>
+      </c>
+    </row>
+    <row r="12" ht="15" customHeight="1">
+      <c r="B12" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  有效稅率（2026E）</t>
+        </is>
+      </c>
+      <c r="F12" s="58" t="n">
+        <v>0.08</v>
+      </c>
+    </row>
+    <row r="13" ht="15" customHeight="1">
+      <c r="B13" s="24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  稅後債務成本</t>
+        </is>
+      </c>
+      <c r="F13" s="65" t="n">
+        <v>0.0534</v>
+      </c>
+    </row>
+    <row r="14" ht="15" customHeight="1">
+      <c r="B14" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  股本比重</t>
+        </is>
+      </c>
+      <c r="F14" s="58" t="n">
+        <v>0.981</v>
+      </c>
+    </row>
+    <row r="15" ht="15" customHeight="1">
+      <c r="B15" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  債務比重</t>
+        </is>
+      </c>
+      <c r="F15" s="58" t="n">
+        <v>0.019</v>
+      </c>
+    </row>
+    <row r="16" ht="15" customHeight="1">
+      <c r="B16" s="24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  WACC（基準）</t>
+        </is>
+      </c>
+      <c r="F16" s="65" t="n">
+        <v>0.135</v>
+      </c>
+    </row>
+    <row r="17" ht="5" customHeight="1"/>
+    <row r="18">
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  無槓桿自由現金流 (UFCF)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="15" customHeight="1">
+      <c r="B19" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  EBIT</t>
+        </is>
+      </c>
+      <c r="C19" s="8" t="n">
+        <v>2748.98</v>
+      </c>
+      <c r="D19" s="8" t="n">
+        <v>6173.1</v>
+      </c>
+      <c r="E19" s="8" t="n">
+        <v>11283.98</v>
+      </c>
+      <c r="F19" s="8" t="n">
+        <v>17775.6</v>
+      </c>
+      <c r="G19" s="8" t="n">
+        <v>25055.38</v>
+      </c>
+    </row>
+    <row r="20" ht="15" customHeight="1">
+      <c r="B20" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  × (1 − 有效稅率)</t>
+        </is>
+      </c>
+      <c r="C20" s="25" t="n">
+        <v>0.92</v>
+      </c>
+      <c r="D20" s="25" t="n">
+        <v>0.88</v>
+      </c>
+      <c r="E20" s="25" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="F20" s="25" t="n">
+        <v>0.83</v>
+      </c>
+      <c r="G20" s="25" t="n">
+        <v>0.82</v>
+      </c>
+    </row>
+    <row r="21" ht="15" customHeight="1">
+      <c r="B21" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  = NOPAT</t>
+        </is>
+      </c>
+      <c r="C21" s="66" t="n">
+        <v>2529.06</v>
+      </c>
+      <c r="D21" s="66" t="n">
+        <v>5432.33</v>
+      </c>
+      <c r="E21" s="66" t="n">
+        <v>9591.379999999999</v>
+      </c>
+      <c r="F21" s="66" t="n">
+        <v>14753.75</v>
+      </c>
+      <c r="G21" s="66" t="n">
+        <v>20545.41</v>
+      </c>
+    </row>
+    <row r="22" ht="15" customHeight="1">
+      <c r="B22" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  + 折舊及攤銷（D&amp;A）</t>
+        </is>
+      </c>
+      <c r="C22" s="8" t="n">
+        <v>2507.4</v>
+      </c>
+      <c r="D22" s="8" t="n">
+        <v>3344</v>
+      </c>
+      <c r="E22" s="8" t="n">
+        <v>4323.1</v>
+      </c>
+      <c r="F22" s="8" t="n">
+        <v>5424.3</v>
+      </c>
+      <c r="G22" s="8" t="n">
+        <v>6550.68</v>
+      </c>
+    </row>
+    <row r="23" ht="15" customHeight="1">
+      <c r="B23" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  − 資本支出（CapEx）</t>
+        </is>
+      </c>
+      <c r="C23" s="8" t="n">
+        <v>-6129.2</v>
+      </c>
+      <c r="D23" s="8" t="n">
+        <v>-7600</v>
+      </c>
+      <c r="E23" s="8" t="n">
+        <v>-9154.799999999999</v>
+      </c>
+      <c r="F23" s="8" t="n">
+        <v>-10584</v>
+      </c>
+      <c r="G23" s="8" t="n">
+        <v>-12438</v>
+      </c>
+    </row>
+    <row r="24" ht="15" customHeight="1">
+      <c r="B24" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  − 營運資本變動（ΔNWC）</t>
+        </is>
+      </c>
+      <c r="C24" s="8" t="n">
+        <v>-417.9</v>
+      </c>
+      <c r="D24" s="8" t="n">
+        <v>-570</v>
+      </c>
+      <c r="E24" s="8" t="n">
+        <v>-762.9</v>
+      </c>
+      <c r="F24" s="8" t="n">
+        <v>-992.25</v>
+      </c>
+      <c r="G24" s="8" t="n">
+        <v>-1243.8</v>
+      </c>
+    </row>
+    <row r="25" ht="15" customHeight="1">
+      <c r="B25" s="24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  = 無槓桿自由現金流（UFCF）</t>
+        </is>
+      </c>
+      <c r="C25" s="28" t="n">
+        <v>-674.84</v>
+      </c>
+      <c r="D25" s="28" t="n">
+        <v>1746.33</v>
+      </c>
+      <c r="E25" s="28" t="n">
+        <v>5522.58</v>
+      </c>
+      <c r="F25" s="28" t="n">
+        <v>10586.3</v>
+      </c>
+      <c r="G25" s="28" t="n">
+        <v>15901.89</v>
+      </c>
+    </row>
+    <row r="26" ht="5" customHeight="1"/>
+    <row r="27">
+      <c r="B27" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  折現計算</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="15" customHeight="1">
+      <c r="B28" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  折現因子 (1/(1+WACC)^t)</t>
+        </is>
+      </c>
+      <c r="C28" s="67" t="n">
+        <v>0.88</v>
+      </c>
+      <c r="D28" s="67" t="n">
+        <v>0.78</v>
+      </c>
+      <c r="E28" s="67" t="n">
+        <v>0.68</v>
+      </c>
+      <c r="F28" s="67" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="G28" s="67" t="n">
+        <v>0.53</v>
+      </c>
+    </row>
+    <row r="29" ht="15" customHeight="1">
+      <c r="B29" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  UFCF 現值 ($M)</t>
+        </is>
+      </c>
+      <c r="C29" s="8" t="n">
+        <v>-594.5700000000001</v>
+      </c>
+      <c r="D29" s="8" t="n">
+        <v>1355.61</v>
+      </c>
+      <c r="E29" s="8" t="n">
+        <v>3777.07</v>
+      </c>
+      <c r="F29" s="8" t="n">
+        <v>6379.12</v>
+      </c>
+      <c r="G29" s="8" t="n">
+        <v>8442.469999999999</v>
+      </c>
+    </row>
+    <row r="30" ht="5" customHeight="1"/>
+    <row r="31">
+      <c r="B31" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  企業價值橋接</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="15" customHeight="1">
+      <c r="B32" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  UFCF 現值合計</t>
+        </is>
+      </c>
+      <c r="F32" s="8" t="n">
+        <v>19359.69</v>
+      </c>
+    </row>
+    <row r="33" ht="15" customHeight="1">
+      <c r="B33" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  2030E EBITDA × 18x 退出倍數（終值）</t>
+        </is>
+      </c>
+      <c r="F33" s="8" t="n">
+        <v>568909.08</v>
+      </c>
+    </row>
+    <row r="34" ht="15" customHeight="1">
+      <c r="B34" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  終值現值 (PV of TV)</t>
+        </is>
+      </c>
+      <c r="F34" s="8" t="n">
+        <v>302039.37</v>
+      </c>
+    </row>
+    <row r="35" ht="15" customHeight="1">
+      <c r="B35" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  終值佔企業價值比重</t>
+        </is>
+      </c>
+      <c r="F35" s="25" t="n">
+        <v>0.9399999999999999</v>
+      </c>
+    </row>
+    <row r="36" ht="15" customHeight="1">
+      <c r="B36" s="24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  企業價值（DCF）</t>
+        </is>
+      </c>
+      <c r="F36" s="28" t="n">
+        <v>321399.06</v>
+      </c>
+    </row>
+    <row r="37" ht="15" customHeight="1">
+      <c r="B37" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  + 淨現金（2026E 末，含 IPO 募資）</t>
+        </is>
+      </c>
+      <c r="F37" s="8" t="n">
+        <v>85322.48</v>
+      </c>
+    </row>
+    <row r="38" ht="15" customHeight="1">
+      <c r="B38" s="24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  股票價值</t>
+        </is>
+      </c>
+      <c r="F38" s="28" t="n">
+        <v>406721.54</v>
+      </c>
+    </row>
+    <row r="39" ht="15" customHeight="1">
+      <c r="B39" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ÷ 攤薄股數（M）</t>
+        </is>
+      </c>
+      <c r="F39" s="8" t="n">
+        <v>2120</v>
+      </c>
+    </row>
+    <row r="40" ht="15" customHeight="1">
+      <c r="B40" s="24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  每股股價（DCF）</t>
+        </is>
+      </c>
+      <c r="F40" s="68" t="n">
+        <v>191.85</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="6">
+    <mergeCell ref="B18:I18"/>
+    <mergeCell ref="B6:I6"/>
+    <mergeCell ref="B2:I2"/>
+    <mergeCell ref="B31:I31"/>
+    <mergeCell ref="B27:I27"/>
+    <mergeCell ref="B1:I1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="002F5496"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="B1:M19"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="2" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="12" customWidth="1" min="13" max="13"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="26" customHeight="1">
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>SpaceX (SPCE)  —  敏感性分析</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="13" customHeight="1">
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>表一：WACC × 退出倍數；表二：收入CAGR × 2030E EBITDA利潤率；單位：美元每股（$/股）</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="5" customHeight="1"/>
+    <row r="5">
+      <c r="B5" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  表一：WACC × 退出 EV/EBITDA 倍數（每股股價 $）</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="B6" s="63" t="inlineStr">
+        <is>
+          <t>WACC \ 退出倍數</t>
+        </is>
+      </c>
+      <c r="C6" s="63" t="inlineStr">
+        <is>
+          <t>14x</t>
+        </is>
+      </c>
+      <c r="D6" s="63" t="inlineStr">
+        <is>
+          <t>16x</t>
+        </is>
+      </c>
+      <c r="E6" s="69" t="inlineStr">
+        <is>
+          <t>18x</t>
+        </is>
+      </c>
+      <c r="F6" s="63" t="inlineStr">
+        <is>
+          <t>20x</t>
+        </is>
+      </c>
+      <c r="G6" s="63" t="inlineStr">
+        <is>
+          <t>22x</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="15" customHeight="1">
+      <c r="B7" s="40" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  11.5%</t>
+        </is>
+      </c>
+      <c r="C7" s="70" t="n">
+        <v>171.2</v>
+      </c>
+      <c r="D7" s="70" t="n">
+        <v>188.5</v>
+      </c>
+      <c r="E7" s="71" t="n">
+        <v>205.8</v>
+      </c>
+      <c r="F7" s="72" t="n">
+        <v>223.1</v>
+      </c>
+      <c r="G7" s="72" t="n">
+        <v>240.41</v>
+      </c>
+    </row>
+    <row r="8" ht="15" customHeight="1">
+      <c r="B8" s="40" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  12.5%</t>
+        </is>
+      </c>
+      <c r="C8" s="73" t="n">
+        <v>165.55</v>
+      </c>
+      <c r="D8" s="70" t="n">
+        <v>182.09</v>
+      </c>
+      <c r="E8" s="71" t="n">
+        <v>198.64</v>
+      </c>
+      <c r="F8" s="71" t="n">
+        <v>215.19</v>
+      </c>
+      <c r="G8" s="72" t="n">
+        <v>231.73</v>
+      </c>
+    </row>
+    <row r="9" ht="15" customHeight="1">
+      <c r="B9" s="74" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  13.5%</t>
+        </is>
+      </c>
+      <c r="C9" s="75" t="n">
+        <v>160.19</v>
+      </c>
+      <c r="D9" s="76" t="n">
+        <v>176.02</v>
+      </c>
+      <c r="E9" s="76" t="n">
+        <v>191.85</v>
+      </c>
+      <c r="F9" s="77" t="n">
+        <v>207.68</v>
+      </c>
+      <c r="G9" s="78" t="n">
+        <v>223.51</v>
+      </c>
+    </row>
+    <row r="10" ht="15" customHeight="1">
+      <c r="B10" s="40" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  14.5%</t>
+        </is>
+      </c>
+      <c r="C10" s="73" t="n">
+        <v>155.1</v>
+      </c>
+      <c r="D10" s="70" t="n">
+        <v>170.26</v>
+      </c>
+      <c r="E10" s="70" t="n">
+        <v>185.41</v>
+      </c>
+      <c r="F10" s="71" t="n">
+        <v>200.56</v>
+      </c>
+      <c r="G10" s="71" t="n">
+        <v>215.71</v>
+      </c>
+    </row>
+    <row r="11" ht="15" customHeight="1">
+      <c r="B11" s="40" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  15.5%</t>
+        </is>
+      </c>
+      <c r="C11" s="73" t="n">
+        <v>150.28</v>
+      </c>
+      <c r="D11" s="73" t="n">
+        <v>164.78</v>
+      </c>
+      <c r="E11" s="70" t="n">
+        <v>179.29</v>
+      </c>
+      <c r="F11" s="71" t="n">
+        <v>193.8</v>
+      </c>
+      <c r="G11" s="71" t="n">
+        <v>208.3</v>
+      </c>
+    </row>
+    <row r="12" ht="10" customHeight="1"/>
+    <row r="13">
+      <c r="B13" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  表二：收入 CAGR × 2030E EBITDA 利潤率（每股股價 $）</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="B14" s="63" t="inlineStr">
+        <is>
+          <t>收入CAGR \ EBITDA率</t>
+        </is>
+      </c>
+      <c r="C14" s="63" t="inlineStr">
+        <is>
+          <t>32%</t>
+        </is>
+      </c>
+      <c r="D14" s="63" t="inlineStr">
+        <is>
+          <t>34%</t>
+        </is>
+      </c>
+      <c r="E14" s="63" t="inlineStr">
+        <is>
+          <t>36%</t>
+        </is>
+      </c>
+      <c r="F14" s="69" t="inlineStr">
+        <is>
+          <t>38%</t>
+        </is>
+      </c>
+      <c r="G14" s="63" t="inlineStr">
+        <is>
+          <t>40%</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="15" customHeight="1">
+      <c r="B15" s="40" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  23%</t>
+        </is>
+      </c>
+      <c r="C15" s="79" t="n">
+        <v>127.14</v>
+      </c>
+      <c r="D15" s="79" t="n">
+        <v>132.19</v>
+      </c>
+      <c r="E15" s="79" t="n">
+        <v>137.23</v>
+      </c>
+      <c r="F15" s="73" t="n">
+        <v>142.28</v>
+      </c>
+      <c r="G15" s="73" t="n">
+        <v>147.33</v>
+      </c>
+    </row>
+    <row r="16" ht="15" customHeight="1">
+      <c r="B16" s="40" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  27%</t>
+        </is>
+      </c>
+      <c r="C16" s="73" t="n">
+        <v>142.22</v>
+      </c>
+      <c r="D16" s="73" t="n">
+        <v>148.14</v>
+      </c>
+      <c r="E16" s="73" t="n">
+        <v>154.06</v>
+      </c>
+      <c r="F16" s="73" t="n">
+        <v>159.99</v>
+      </c>
+      <c r="G16" s="73" t="n">
+        <v>165.91</v>
+      </c>
+    </row>
+    <row r="17" ht="15" customHeight="1">
+      <c r="B17" s="74" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  31%</t>
+        </is>
+      </c>
+      <c r="C17" s="75" t="n">
+        <v>159.32</v>
+      </c>
+      <c r="D17" s="75" t="n">
+        <v>166.24</v>
+      </c>
+      <c r="E17" s="76" t="n">
+        <v>173.15</v>
+      </c>
+      <c r="F17" s="76" t="n">
+        <v>180.07</v>
+      </c>
+      <c r="G17" s="76" t="n">
+        <v>186.98</v>
+      </c>
+    </row>
+    <row r="18" ht="15" customHeight="1">
+      <c r="B18" s="40" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  35%</t>
+        </is>
+      </c>
+      <c r="C18" s="70" t="n">
+        <v>178.65</v>
+      </c>
+      <c r="D18" s="70" t="n">
+        <v>186.69</v>
+      </c>
+      <c r="E18" s="70" t="n">
+        <v>194.72</v>
+      </c>
+      <c r="F18" s="71" t="n">
+        <v>202.76</v>
+      </c>
+      <c r="G18" s="71" t="n">
+        <v>210.8</v>
+      </c>
+    </row>
+    <row r="19" ht="15" customHeight="1">
+      <c r="B19" s="40" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  39%</t>
+        </is>
+      </c>
+      <c r="C19" s="71" t="n">
+        <v>200.41</v>
+      </c>
+      <c r="D19" s="71" t="n">
+        <v>209.7</v>
+      </c>
+      <c r="E19" s="71" t="n">
+        <v>219</v>
+      </c>
+      <c r="F19" s="71" t="n">
+        <v>228.3</v>
+      </c>
+      <c r="G19" s="71" t="n">
+        <v>237.6</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="4">
+    <mergeCell ref="B13:I13"/>
+    <mergeCell ref="B2:M2"/>
+    <mergeCell ref="B5:I5"/>
+    <mergeCell ref="B1:M1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="00375623"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="B1:J25"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="2" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="8" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="11" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="11" customWidth="1" min="8" max="8"/>
+    <col width="11" customWidth="1" min="9" max="9"/>
+    <col width="10" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="26" customHeight="1">
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>SpaceX (SPCE)  —  可比公司分析</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="13" customHeight="1">
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>市場數據截至 2026年5月23日；NTM = 2027E；$B = 十億美元；來源：彭博、FactSet、公司公告</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="5" customHeight="1"/>
+    <row r="5" ht="28" customHeight="1">
+      <c r="B5" s="63" t="inlineStr">
+        <is>
+          <t>公司</t>
+        </is>
+      </c>
+      <c r="C5" s="63" t="inlineStr">
+        <is>
+          <t>代號</t>
+        </is>
+      </c>
+      <c r="D5" s="63" t="inlineStr">
+        <is>
+          <t>市值($B)</t>
+        </is>
+      </c>
+      <c r="E5" s="63" t="inlineStr">
+        <is>
+          <t>EV($B)</t>
+        </is>
+      </c>
+      <c r="F5" s="63" t="inlineStr">
+        <is>
+          <t>EV/NTM
+收入</t>
+        </is>
+      </c>
+      <c r="G5" s="63" t="inlineStr">
+        <is>
+          <t>EV/NTM
+EBITDA</t>
+        </is>
+      </c>
+      <c r="H5" s="63" t="inlineStr">
+        <is>
+          <t>NTM收入
+增長</t>
+        </is>
+      </c>
+      <c r="I5" s="63" t="inlineStr">
+        <is>
+          <t>EBITDA
+利潤率</t>
+        </is>
+      </c>
+      <c r="J5" s="63" t="inlineStr">
+        <is>
+          <t>備注</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="14" customHeight="1">
+      <c r="B6" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ── 太空發射 ──</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="16" customHeight="1">
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Rocket Lab</t>
+        </is>
+      </c>
+      <c r="C7" s="40" t="inlineStr">
+        <is>
+          <t>RKLB</t>
+        </is>
+      </c>
+      <c r="D7" s="80" t="n">
+        <v>12.4</v>
+      </c>
+      <c r="E7" s="80" t="n">
+        <v>13.1</v>
+      </c>
+      <c r="F7" s="81" t="n">
+        <v>9.4</v>
+      </c>
+      <c r="G7" s="82" t="inlineStr">
+        <is>
+          <t>n/m</t>
+        </is>
+      </c>
+      <c r="H7" s="25" t="n">
+        <v>0.42</v>
+      </c>
+      <c r="I7" s="25" t="n">
+        <v>-0.12</v>
+      </c>
+      <c r="J7" s="83" t="inlineStr">
+        <is>
+          <t>純發射業務最佳對標</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="16" customHeight="1">
+      <c r="B8" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Northrop Grumman</t>
+        </is>
+      </c>
+      <c r="C8" s="40" t="inlineStr">
+        <is>
+          <t>NOC</t>
+        </is>
+      </c>
+      <c r="D8" s="80" t="n">
+        <v>72.09999999999999</v>
+      </c>
+      <c r="E8" s="80" t="n">
+        <v>78.5</v>
+      </c>
+      <c r="F8" s="81" t="n">
+        <v>1.9</v>
+      </c>
+      <c r="G8" s="81" t="n">
+        <v>12.1</v>
+      </c>
+      <c r="H8" s="25" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="I8" s="25" t="n">
+        <v>0.16</v>
+      </c>
+      <c r="J8" s="83" t="inlineStr">
+        <is>
+          <t>國防/太空系統整合商</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="16" customHeight="1">
+      <c r="B9" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Lockheed Martin</t>
+        </is>
+      </c>
+      <c r="C9" s="40" t="inlineStr">
+        <is>
+          <t>LMT</t>
+        </is>
+      </c>
+      <c r="D9" s="80" t="n">
+        <v>108.3</v>
+      </c>
+      <c r="E9" s="80" t="n">
+        <v>112.8</v>
+      </c>
+      <c r="F9" s="81" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="G9" s="81" t="n">
+        <v>11.3</v>
+      </c>
+      <c r="H9" s="25" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="I9" s="25" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="J9" s="83" t="inlineStr">
+        <is>
+          <t>國防航太巨頭</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="14" customHeight="1">
+      <c r="B10" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ── 衛星連接 ──</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="16" customHeight="1">
+      <c r="B11" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Viasat</t>
+        </is>
+      </c>
+      <c r="C11" s="40" t="inlineStr">
+        <is>
+          <t>VSAT</t>
+        </is>
+      </c>
+      <c r="D11" s="80" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="E11" s="80" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="F11" s="81" t="n">
+        <v>2</v>
+      </c>
+      <c r="G11" s="81" t="n">
+        <v>7.8</v>
+      </c>
+      <c r="H11" s="25" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="I11" s="25" t="n">
+        <v>0.26</v>
+      </c>
+      <c r="J11" s="83" t="inlineStr">
+        <is>
+          <t>衛星寬頻服務商</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="16" customHeight="1">
+      <c r="B12" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Iridium</t>
+        </is>
+      </c>
+      <c r="C12" s="40" t="inlineStr">
+        <is>
+          <t>IRDM</t>
+        </is>
+      </c>
+      <c r="D12" s="80" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="E12" s="80" t="n">
+        <v>5.2</v>
+      </c>
+      <c r="F12" s="81" t="n">
+        <v>6.5</v>
+      </c>
+      <c r="G12" s="81" t="n">
+        <v>10.4</v>
+      </c>
+      <c r="H12" s="25" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="I12" s="25" t="n">
+        <v>0.62</v>
+      </c>
+      <c r="J12" s="83" t="inlineStr">
+        <is>
+          <t>低軌衛星連接</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="16" customHeight="1">
+      <c r="B13" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  AST SpaceMobile</t>
+        </is>
+      </c>
+      <c r="C13" s="40" t="inlineStr">
+        <is>
+          <t>ASTS</t>
+        </is>
+      </c>
+      <c r="D13" s="80" t="n">
+        <v>14.2</v>
+      </c>
+      <c r="E13" s="80" t="n">
+        <v>14.5</v>
+      </c>
+      <c r="F13" s="82" t="inlineStr">
+        <is>
+          <t>n/m</t>
+        </is>
+      </c>
+      <c r="G13" s="82" t="inlineStr">
+        <is>
+          <t>n/m</t>
+        </is>
+      </c>
+      <c r="H13" s="25" t="n">
+        <v>1.82</v>
+      </c>
+      <c r="I13" s="82" t="inlineStr">
+        <is>
+          <t>n/m</t>
+        </is>
+      </c>
+      <c r="J13" s="83" t="inlineStr">
+        <is>
+          <t>直連手機衛星新興股</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="14" customHeight="1">
+      <c r="B14" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ── AI/科技/防禦 ──</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="16" customHeight="1">
+      <c r="B15" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Palantir</t>
+        </is>
+      </c>
+      <c r="C15" s="40" t="inlineStr">
+        <is>
+          <t>PLTR</t>
+        </is>
+      </c>
+      <c r="D15" s="80" t="n">
+        <v>139.8</v>
+      </c>
+      <c r="E15" s="80" t="n">
+        <v>137.4</v>
+      </c>
+      <c r="F15" s="81" t="n">
+        <v>28.6</v>
+      </c>
+      <c r="G15" s="82" t="inlineStr">
+        <is>
+          <t>n/m</t>
+        </is>
+      </c>
+      <c r="H15" s="25" t="n">
+        <v>0.32</v>
+      </c>
+      <c r="I15" s="25" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="J15" s="83" t="inlineStr">
+        <is>
+          <t>AI/政府科技最高增長估值</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="16" customHeight="1">
+      <c r="B16" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  L3 Harris</t>
+        </is>
+      </c>
+      <c r="C16" s="40" t="inlineStr">
+        <is>
+          <t>LHX</t>
+        </is>
+      </c>
+      <c r="D16" s="80" t="n">
+        <v>40.2</v>
+      </c>
+      <c r="E16" s="80" t="n">
+        <v>43.8</v>
+      </c>
+      <c r="F16" s="81" t="n">
+        <v>2.1</v>
+      </c>
+      <c r="G16" s="81" t="n">
+        <v>13.2</v>
+      </c>
+      <c r="H16" s="25" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="I16" s="25" t="n">
+        <v>0.16</v>
+      </c>
+      <c r="J16" s="83" t="inlineStr">
+        <is>
+          <t>國防電子/太空</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="5" customHeight="1"/>
+    <row r="18" ht="18" customHeight="1">
+      <c r="B18" s="84" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  SpaceX</t>
+        </is>
+      </c>
+      <c r="C18" s="85" t="inlineStr">
+        <is>
+          <t>SPCE</t>
+        </is>
+      </c>
+      <c r="D18" s="86" t="n">
+        <v>322.2</v>
+      </c>
+      <c r="E18" s="87" t="inlineStr">
+        <is>
+          <t>估算</t>
+        </is>
+      </c>
+      <c r="F18" s="88" t="n">
+        <v>9</v>
+      </c>
+      <c r="G18" s="88" t="n">
+        <v>35.9</v>
+      </c>
+      <c r="H18" s="89" t="n">
+        <v>0.36</v>
+      </c>
+      <c r="I18" s="89" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="J18" s="90" t="inlineStr">
+        <is>
+          <t>目標倍數（業務組合溢價）</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="8" customHeight="1"/>
+    <row r="20">
+      <c r="B20" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  統計摘要</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="15" customHeight="1">
+      <c r="B21" s="91" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  最高值</t>
+        </is>
+      </c>
+      <c r="C21" s="92" t="n"/>
+      <c r="D21" s="92" t="n"/>
+      <c r="E21" s="92" t="n"/>
+      <c r="F21" s="93" t="n">
+        <v>28.6</v>
+      </c>
+      <c r="G21" s="93" t="n">
+        <v>13.2</v>
+      </c>
+      <c r="H21" s="94" t="n">
+        <v>1.82</v>
+      </c>
+      <c r="I21" s="94" t="n">
+        <v>0.62</v>
+      </c>
+    </row>
+    <row r="22" ht="15" customHeight="1">
+      <c r="B22" s="91" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  75百分位</t>
+        </is>
+      </c>
+      <c r="C22" s="92" t="n"/>
+      <c r="D22" s="92" t="n"/>
+      <c r="E22" s="92" t="n"/>
+      <c r="F22" s="93" t="n">
+        <v>7.95</v>
+      </c>
+      <c r="G22" s="93" t="n">
+        <v>12.1</v>
+      </c>
+      <c r="H22" s="94" t="n">
+        <v>0.345</v>
+      </c>
+      <c r="I22" s="94" t="n">
+        <v>0.27</v>
+      </c>
+    </row>
+    <row r="23" ht="15" customHeight="1">
+      <c r="B23" s="95" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  中位數</t>
+        </is>
+      </c>
+      <c r="C23" s="96" t="n"/>
+      <c r="D23" s="96" t="n"/>
+      <c r="E23" s="96" t="n"/>
+      <c r="F23" s="97" t="n">
+        <v>2.1</v>
+      </c>
+      <c r="G23" s="97" t="n">
+        <v>11.3</v>
+      </c>
+      <c r="H23" s="98" t="n">
+        <v>0.065</v>
+      </c>
+      <c r="I23" s="98" t="n">
+        <v>0.16</v>
+      </c>
+    </row>
+    <row r="24" ht="15" customHeight="1">
+      <c r="B24" s="91" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  25百分位</t>
+        </is>
+      </c>
+      <c r="C24" s="92" t="n"/>
+      <c r="D24" s="92" t="n"/>
+      <c r="E24" s="92" t="n"/>
+      <c r="F24" s="93" t="n">
+        <v>1.95</v>
+      </c>
+      <c r="G24" s="93" t="n">
+        <v>10.4</v>
+      </c>
+      <c r="H24" s="94" t="n">
+        <v>0.0475</v>
+      </c>
+      <c r="I24" s="94" t="n">
+        <v>0.155</v>
+      </c>
+    </row>
+    <row r="25" ht="15" customHeight="1">
+      <c r="B25" s="91" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  最低值</t>
+        </is>
+      </c>
+      <c r="C25" s="92" t="n"/>
+      <c r="D25" s="92" t="n"/>
+      <c r="E25" s="92" t="n"/>
+      <c r="F25" s="93" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="G25" s="93" t="n">
+        <v>7.8</v>
+      </c>
+      <c r="H25" s="94" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="I25" s="94" t="n">
+        <v>-0.12</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="6">
+    <mergeCell ref="B20:J20"/>
+    <mergeCell ref="B10:J10"/>
+    <mergeCell ref="B14:J14"/>
+    <mergeCell ref="B1:J1"/>
+    <mergeCell ref="B6:J6"/>
+    <mergeCell ref="B2:J2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>